<commit_message>
completati criteri di Bears
</commit_message>
<xml_diff>
--- a/i_test/test_D3_coorte_con_bears/med_anticol.xlsx
+++ b/i_test/test_D3_coorte_con_bears/med_anticol.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="11">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -257,7 +257,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
@@ -305,7 +305,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>20251231</v>
+        <v>20251226</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>7</v>
@@ -313,26 +313,26 @@
       <c r="D4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>20251010</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="4"/>
+      <c r="A5" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>20251231</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="4" t="n">
-        <v>20251024</v>
+        <v>20251010</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -341,34 +341,34 @@
         <v>8</v>
       </c>
       <c r="B7" s="4" t="n">
-        <v>20241110</v>
+        <v>20251023</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>20251024</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="4"/>
-    </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>20251010</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="5"/>
+      <c r="D8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>20251024</v>
+        <v>20241222</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D9" s="5"/>
     </row>
@@ -377,12 +377,24 @@
         <v>10</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>20241108</v>
+        <v>20250105</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="5"/>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>20250108</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="5"/>
+      <c r="D11" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>